<commit_message>
Organised the URLs into config folder
</commit_message>
<xml_diff>
--- a/output/cfr_scopus_mjl_scimago_results.xlsx
+++ b/output/cfr_scopus_mjl_scimago_results.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="n">
-        <v>1.5</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="3">
@@ -797,7 +797,7 @@
       </c>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="n">
-        <v>1.31</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="4">
@@ -919,7 +919,7 @@
       </c>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="n">
-        <v>1.17</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="5">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="n">
-        <v>1.06</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="6">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="n">
-        <v>1.19</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="7">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="n">
-        <v>1.07</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="8">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="n">
-        <v>0.99</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="9">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="n">
-        <v>1.25</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="10">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="n">
-        <v>1.46</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="11">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="n">
-        <v>1.3</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="12">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="n">
-        <v>1.42</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="13">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="n">
-        <v>1.39</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="14">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="n">
-        <v>1.45</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="15">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="n">
-        <v>1.46</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="16">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="n">
-        <v>1.44</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="17">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="n">
-        <v>1.45</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="18">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="n">
-        <v>1.45</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="19">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="n">
-        <v>1.45</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="20">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="n">
-        <v>1.43</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="21">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="n">
-        <v>1.45</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="22">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="n">
-        <v>1.42</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="n">
-        <v>1.4</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="24">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="n">
-        <v>1.47</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="25">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="n">
-        <v>1.43</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="26">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="n">
-        <v>1.43</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="27">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="n">
-        <v>1.42</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="28">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="n">
-        <v>1.42</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="29">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="n">
-        <v>1.45</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="30">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="n">
-        <v>1.41</v>
+        <v>4.36</v>
       </c>
     </row>
     <row r="31">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="n">
-        <v>1.45</v>
+        <v>4.33</v>
       </c>
     </row>
     <row r="32">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="n">
-        <v>1.43</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="33">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="n">
-        <v>1.43</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="34">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="n">
-        <v>1.43</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="35">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="n">
-        <v>1.46</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="36">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="n">
-        <v>1.41</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="37">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="n">
-        <v>1.44</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="38">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="n">
-        <v>1.43</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="39">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="n">
-        <v>1.44</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="40">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="n">
-        <v>1.44</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="41">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="n">
-        <v>1.46</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="42">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="n">
-        <v>1.46</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="43">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="n">
-        <v>1.45</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="44">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="n">
-        <v>1.48</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="45">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="Y45" t="inlineStr"/>
       <c r="Z45" t="n">
-        <v>1.44</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="46">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="n">
-        <v>1.44</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="47">
@@ -6269,7 +6269,7 @@
       </c>
       <c r="Y47" t="inlineStr"/>
       <c r="Z47" t="n">
-        <v>1.47</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="48">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="n">
-        <v>1.41</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="49">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="Y49" t="inlineStr"/>
       <c r="Z49" t="n">
-        <v>1.45</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="50">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="n">
-        <v>1.43</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="51">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="n">
-        <v>1.44</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="52">
@@ -6899,7 +6899,7 @@
       </c>
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="n">
-        <v>1.41</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="53">
@@ -7025,7 +7025,7 @@
       </c>
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="n">
-        <v>1.46</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="54">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="n">
-        <v>1.44</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="55">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="n">
-        <v>1.48</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="56">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="Y56" t="inlineStr"/>
       <c r="Z56" t="n">
-        <v>1.73</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="57">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="Y57" t="inlineStr"/>
       <c r="Z57" t="n">
-        <v>1.54</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="58">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="Y58" t="inlineStr"/>
       <c r="Z58" t="n">
-        <v>1.49</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="59">
@@ -7769,7 +7769,7 @@
       </c>
       <c r="Y59" t="inlineStr"/>
       <c r="Z59" t="n">
-        <v>1.4</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="60">
@@ -7895,7 +7895,7 @@
       </c>
       <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="n">
-        <v>1.43</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="61">
@@ -8017,7 +8017,7 @@
       </c>
       <c r="Y61" t="inlineStr"/>
       <c r="Z61" t="n">
-        <v>1.44</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="62">
@@ -8139,7 +8139,7 @@
       </c>
       <c r="Y62" t="inlineStr"/>
       <c r="Z62" t="n">
-        <v>1.45</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="63">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="Y63" t="inlineStr"/>
       <c r="Z63" t="n">
-        <v>1.45</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="64">
@@ -8391,7 +8391,7 @@
       </c>
       <c r="Y64" t="inlineStr"/>
       <c r="Z64" t="n">
-        <v>1.44</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="65">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="Y65" t="inlineStr"/>
       <c r="Z65" t="n">
-        <v>1.43</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="66">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="Y66" t="inlineStr"/>
       <c r="Z66" t="n">
-        <v>1.42</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="67">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="Y67" t="inlineStr"/>
       <c r="Z67" t="n">
-        <v>1.45</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="68">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="Y68" t="inlineStr"/>
       <c r="Z68" t="n">
-        <v>1.47</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="69">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="Y69" t="inlineStr"/>
       <c r="Z69" t="n">
-        <v>1.5</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="70">
@@ -9143,7 +9143,7 @@
       </c>
       <c r="Y70" t="inlineStr"/>
       <c r="Z70" t="n">
-        <v>1.45</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="71">
@@ -9265,7 +9265,7 @@
       </c>
       <c r="Y71" t="inlineStr"/>
       <c r="Z71" t="n">
-        <v>1.45</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="72">
@@ -9391,7 +9391,7 @@
       </c>
       <c r="Y72" t="inlineStr"/>
       <c r="Z72" t="n">
-        <v>1.44</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="73">
@@ -9517,7 +9517,7 @@
       </c>
       <c r="Y73" t="inlineStr"/>
       <c r="Z73" t="n">
-        <v>1.44</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="74">
@@ -9643,7 +9643,7 @@
       </c>
       <c r="Y74" t="inlineStr"/>
       <c r="Z74" t="n">
-        <v>1.45</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="75">
@@ -9769,7 +9769,7 @@
       </c>
       <c r="Y75" t="inlineStr"/>
       <c r="Z75" t="n">
-        <v>1.43</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="76">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="Y76" t="inlineStr"/>
       <c r="Z76" t="n">
-        <v>1.47</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="77">
@@ -10013,7 +10013,7 @@
       </c>
       <c r="Y77" t="inlineStr"/>
       <c r="Z77" t="n">
-        <v>1.49</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="78">
@@ -10139,7 +10139,7 @@
       </c>
       <c r="Y78" t="inlineStr"/>
       <c r="Z78" t="n">
-        <v>1.49</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="79">
@@ -10265,7 +10265,7 @@
       </c>
       <c r="Y79" t="inlineStr"/>
       <c r="Z79" t="n">
-        <v>1.43</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="80">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="Y80" t="inlineStr"/>
       <c r="Z80" t="n">
-        <v>1.45</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="81">
@@ -10517,7 +10517,7 @@
       </c>
       <c r="Y81" t="inlineStr"/>
       <c r="Z81" t="n">
-        <v>1.45</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="82">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="Y82" t="inlineStr"/>
       <c r="Z82" t="n">
-        <v>1.48</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="83">
@@ -10769,7 +10769,7 @@
       </c>
       <c r="Y83" t="inlineStr"/>
       <c r="Z83" t="n">
-        <v>1.48</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="84">
@@ -10895,7 +10895,7 @@
       </c>
       <c r="Y84" t="inlineStr"/>
       <c r="Z84" t="n">
-        <v>1.39</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="85">
@@ -11021,7 +11021,7 @@
       </c>
       <c r="Y85" t="inlineStr"/>
       <c r="Z85" t="n">
-        <v>1.41</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="86">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="Y86" t="inlineStr"/>
       <c r="Z86" t="n">
-        <v>1.43</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="87">
@@ -11269,7 +11269,7 @@
       </c>
       <c r="Y87" t="inlineStr"/>
       <c r="Z87" t="n">
-        <v>1.42</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="88">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="Y88" t="inlineStr"/>
       <c r="Z88" t="n">
-        <v>1.45</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="89">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="Y89" t="inlineStr"/>
       <c r="Z89" t="n">
-        <v>1.42</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="90">
@@ -11639,7 +11639,7 @@
       </c>
       <c r="Y90" t="inlineStr"/>
       <c r="Z90" t="n">
-        <v>1.45</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="91">
@@ -11761,7 +11761,7 @@
       </c>
       <c r="Y91" t="inlineStr"/>
       <c r="Z91" t="n">
-        <v>1.45</v>
+        <v>2.87</v>
       </c>
     </row>
     <row r="92">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="Y92" t="inlineStr"/>
       <c r="Z92" t="n">
-        <v>1.44</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="93">
@@ -12013,7 +12013,7 @@
       </c>
       <c r="Y93" t="inlineStr"/>
       <c r="Z93" t="n">
-        <v>1.45</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="94">
@@ -12135,7 +12135,7 @@
       </c>
       <c r="Y94" t="inlineStr"/>
       <c r="Z94" t="n">
-        <v>1.45</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="95">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="Y95" t="inlineStr"/>
       <c r="Z95" t="n">
-        <v>1.43</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="96">
@@ -12387,7 +12387,7 @@
       </c>
       <c r="Y96" t="inlineStr"/>
       <c r="Z96" t="n">
-        <v>1.44</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="97">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="Y97" t="inlineStr"/>
       <c r="Z97" t="n">
-        <v>1.45</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="98">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="Y98" t="inlineStr"/>
       <c r="Z98" t="n">
-        <v>1.43</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="99">
@@ -12765,7 +12765,7 @@
       </c>
       <c r="Y99" t="inlineStr"/>
       <c r="Z99" t="n">
-        <v>1.44</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="100">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="Y100" t="inlineStr"/>
       <c r="Z100" t="n">
-        <v>1.43</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="101">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="Y101" t="inlineStr"/>
       <c r="Z101" t="n">
-        <v>1.51</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="102">
@@ -13143,7 +13143,7 @@
       </c>
       <c r="Y102" t="inlineStr"/>
       <c r="Z102" t="n">
-        <v>1.48</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="103">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="Y103" t="inlineStr"/>
       <c r="Z103" t="n">
-        <v>1.44</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="104">
@@ -13395,7 +13395,7 @@
       </c>
       <c r="Y104" t="inlineStr"/>
       <c r="Z104" t="n">
-        <v>1.42</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="105">
@@ -13521,7 +13521,7 @@
       </c>
       <c r="Y105" t="inlineStr"/>
       <c r="Z105" t="n">
-        <v>1.44</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="106">
@@ -13643,7 +13643,7 @@
       </c>
       <c r="Y106" t="inlineStr"/>
       <c r="Z106" t="n">
-        <v>1.44</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="107">
@@ -13769,7 +13769,7 @@
       </c>
       <c r="Y107" t="inlineStr"/>
       <c r="Z107" t="n">
-        <v>1.49</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="108">
@@ -13895,7 +13895,7 @@
       </c>
       <c r="Y108" t="inlineStr"/>
       <c r="Z108" t="n">
-        <v>1.42</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="109">
@@ -14021,7 +14021,7 @@
       </c>
       <c r="Y109" t="inlineStr"/>
       <c r="Z109" t="n">
-        <v>1.46</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="110">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="Y110" t="inlineStr"/>
       <c r="Z110" t="n">
-        <v>1.48</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="111">
@@ -14269,7 +14269,7 @@
       </c>
       <c r="Y111" t="inlineStr"/>
       <c r="Z111" t="n">
-        <v>1.47</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="112">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="Y112" t="inlineStr"/>
       <c r="Z112" t="n">
-        <v>1.43</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="113">
@@ -14521,7 +14521,7 @@
       </c>
       <c r="Y113" t="inlineStr"/>
       <c r="Z113" t="n">
-        <v>1.43</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="114">
@@ -14647,7 +14647,7 @@
       </c>
       <c r="Y114" t="inlineStr"/>
       <c r="Z114" t="n">
-        <v>1.41</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="115">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="Y115" t="inlineStr"/>
       <c r="Z115" t="n">
-        <v>1.4</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="116">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="Y116" t="inlineStr"/>
       <c r="Z116" t="n">
-        <v>1.44</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="117">
@@ -15025,7 +15025,7 @@
       </c>
       <c r="Y117" t="inlineStr"/>
       <c r="Z117" t="n">
-        <v>1.45</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="118">
@@ -15151,7 +15151,7 @@
       </c>
       <c r="Y118" t="inlineStr"/>
       <c r="Z118" t="n">
-        <v>1.45</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="119">
@@ -15273,7 +15273,7 @@
       </c>
       <c r="Y119" t="inlineStr"/>
       <c r="Z119" t="n">
-        <v>1.46</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="120">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="Y120" t="inlineStr"/>
       <c r="Z120" t="n">
-        <v>1.42</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="121">
@@ -15525,7 +15525,7 @@
       </c>
       <c r="Y121" t="inlineStr"/>
       <c r="Z121" t="n">
-        <v>1.46</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="122">
@@ -15651,7 +15651,7 @@
       </c>
       <c r="Y122" t="inlineStr"/>
       <c r="Z122" t="n">
-        <v>1.43</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="123">
@@ -15777,7 +15777,7 @@
       </c>
       <c r="Y123" t="inlineStr"/>
       <c r="Z123" t="n">
-        <v>1.4</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="124">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="Y124" t="inlineStr"/>
       <c r="Z124" t="n">
-        <v>1.45</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="125">
@@ -16025,7 +16025,7 @@
       </c>
       <c r="Y125" t="inlineStr"/>
       <c r="Z125" t="n">
-        <v>1.43</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="126">
@@ -16151,7 +16151,7 @@
       </c>
       <c r="Y126" t="inlineStr"/>
       <c r="Z126" t="n">
-        <v>1.44</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="127">
@@ -16277,7 +16277,7 @@
       </c>
       <c r="Y127" t="inlineStr"/>
       <c r="Z127" t="n">
-        <v>1.45</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="128">
@@ -16403,7 +16403,7 @@
       </c>
       <c r="Y128" t="inlineStr"/>
       <c r="Z128" t="n">
-        <v>1.43</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="129">
@@ -16525,7 +16525,7 @@
       </c>
       <c r="Y129" t="inlineStr"/>
       <c r="Z129" t="n">
-        <v>1.43</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="130">
@@ -16647,7 +16647,7 @@
       </c>
       <c r="Y130" t="inlineStr"/>
       <c r="Z130" t="n">
-        <v>1.45</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="131">
@@ -16769,7 +16769,7 @@
       </c>
       <c r="Y131" t="inlineStr"/>
       <c r="Z131" t="n">
-        <v>1.42</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="132">
@@ -16895,7 +16895,7 @@
       </c>
       <c r="Y132" t="inlineStr"/>
       <c r="Z132" t="n">
-        <v>1.44</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="133">
@@ -17017,7 +17017,7 @@
       </c>
       <c r="Y133" t="inlineStr"/>
       <c r="Z133" t="n">
-        <v>1.43</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="134">
@@ -17139,7 +17139,7 @@
       </c>
       <c r="Y134" t="inlineStr"/>
       <c r="Z134" t="n">
-        <v>1.46</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="135">
@@ -17261,7 +17261,7 @@
       </c>
       <c r="Y135" t="inlineStr"/>
       <c r="Z135" t="n">
-        <v>1.46</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="136">
@@ -17383,7 +17383,7 @@
       </c>
       <c r="Y136" t="inlineStr"/>
       <c r="Z136" t="n">
-        <v>1.44</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="137">
@@ -17509,7 +17509,7 @@
       </c>
       <c r="Y137" t="inlineStr"/>
       <c r="Z137" t="n">
-        <v>1.45</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="138">
@@ -17635,7 +17635,7 @@
       </c>
       <c r="Y138" t="inlineStr"/>
       <c r="Z138" t="n">
-        <v>1.44</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="139">
@@ -17757,7 +17757,7 @@
       </c>
       <c r="Y139" t="inlineStr"/>
       <c r="Z139" t="n">
-        <v>1.44</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="140">
@@ -17883,7 +17883,7 @@
       </c>
       <c r="Y140" t="inlineStr"/>
       <c r="Z140" t="n">
-        <v>1.51</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="141">
@@ -18009,7 +18009,7 @@
       </c>
       <c r="Y141" t="inlineStr"/>
       <c r="Z141" t="n">
-        <v>1.53</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="142">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="Y142" t="inlineStr"/>
       <c r="Z142" t="n">
-        <v>1.51</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="143">
@@ -18261,7 +18261,7 @@
       </c>
       <c r="Y143" t="inlineStr"/>
       <c r="Z143" t="n">
-        <v>1.56</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="144">
@@ -18383,7 +18383,7 @@
       </c>
       <c r="Y144" t="inlineStr"/>
       <c r="Z144" t="n">
-        <v>1.51</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="145">
@@ -18509,7 +18509,7 @@
       </c>
       <c r="Y145" t="inlineStr"/>
       <c r="Z145" t="n">
-        <v>1.41</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="146">
@@ -18635,7 +18635,7 @@
       </c>
       <c r="Y146" t="inlineStr"/>
       <c r="Z146" t="n">
-        <v>1.46</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="147">
@@ -18761,7 +18761,7 @@
       </c>
       <c r="Y147" t="inlineStr"/>
       <c r="Z147" t="n">
-        <v>1.42</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="148">
@@ -18883,7 +18883,7 @@
       </c>
       <c r="Y148" t="inlineStr"/>
       <c r="Z148" t="n">
-        <v>1.41</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="149">
@@ -19009,7 +19009,7 @@
       </c>
       <c r="Y149" t="inlineStr"/>
       <c r="Z149" t="n">
-        <v>1.5</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="150">
@@ -19135,7 +19135,7 @@
       </c>
       <c r="Y150" t="inlineStr"/>
       <c r="Z150" t="n">
-        <v>2.78</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="151">
@@ -19261,7 +19261,7 @@
       </c>
       <c r="Y151" t="inlineStr"/>
       <c r="Z151" t="n">
-        <v>1.47</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="152">
@@ -19387,7 +19387,7 @@
       </c>
       <c r="Y152" t="inlineStr"/>
       <c r="Z152" t="n">
-        <v>1.48</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="153">
@@ -19513,7 +19513,7 @@
       </c>
       <c r="Y153" t="inlineStr"/>
       <c r="Z153" t="n">
-        <v>1.44</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="154">
@@ -19635,7 +19635,7 @@
       </c>
       <c r="Y154" t="inlineStr"/>
       <c r="Z154" t="n">
-        <v>1.44</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="155">
@@ -19761,7 +19761,7 @@
       </c>
       <c r="Y155" t="inlineStr"/>
       <c r="Z155" t="n">
-        <v>1.47</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="156">
@@ -19883,7 +19883,7 @@
       </c>
       <c r="Y156" t="inlineStr"/>
       <c r="Z156" t="n">
-        <v>1.45</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="157">
@@ -20009,7 +20009,7 @@
       </c>
       <c r="Y157" t="inlineStr"/>
       <c r="Z157" t="n">
-        <v>1.44</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="158">
@@ -20135,7 +20135,7 @@
       </c>
       <c r="Y158" t="inlineStr"/>
       <c r="Z158" t="n">
-        <v>1.41</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="159">
@@ -20261,7 +20261,7 @@
       </c>
       <c r="Y159" t="inlineStr"/>
       <c r="Z159" t="n">
-        <v>1.43</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="160">
@@ -20383,7 +20383,7 @@
       </c>
       <c r="Y160" t="inlineStr"/>
       <c r="Z160" t="n">
-        <v>1.39</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="161">
@@ -20509,7 +20509,7 @@
       </c>
       <c r="Y161" t="inlineStr"/>
       <c r="Z161" t="n">
-        <v>1.43</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="162">
@@ -20635,7 +20635,7 @@
       </c>
       <c r="Y162" t="inlineStr"/>
       <c r="Z162" t="n">
-        <v>1.44</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="163">
@@ -20761,7 +20761,7 @@
       </c>
       <c r="Y163" t="inlineStr"/>
       <c r="Z163" t="n">
-        <v>1.48</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="164">
@@ -20887,7 +20887,7 @@
       </c>
       <c r="Y164" t="inlineStr"/>
       <c r="Z164" t="n">
-        <v>1.42</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="165">
@@ -21013,7 +21013,7 @@
       </c>
       <c r="Y165" t="inlineStr"/>
       <c r="Z165" t="n">
-        <v>1.49</v>
+        <v>4.98</v>
       </c>
     </row>
     <row r="166">
@@ -21139,7 +21139,7 @@
       </c>
       <c r="Y166" t="inlineStr"/>
       <c r="Z166" t="n">
-        <v>1.49</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="167">
@@ -21265,7 +21265,7 @@
       </c>
       <c r="Y167" t="inlineStr"/>
       <c r="Z167" t="n">
-        <v>1.44</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="168">
@@ -21391,7 +21391,7 @@
       </c>
       <c r="Y168" t="inlineStr"/>
       <c r="Z168" t="n">
-        <v>1.42</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="169">
@@ -21517,7 +21517,7 @@
       </c>
       <c r="Y169" t="inlineStr"/>
       <c r="Z169" t="n">
-        <v>1.44</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="170">
@@ -21643,7 +21643,7 @@
       </c>
       <c r="Y170" t="inlineStr"/>
       <c r="Z170" t="n">
-        <v>2.33</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="171">
@@ -21765,7 +21765,7 @@
       </c>
       <c r="Y171" t="inlineStr"/>
       <c r="Z171" t="n">
-        <v>1.9</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="172">
@@ -21891,7 +21891,7 @@
       </c>
       <c r="Y172" t="inlineStr"/>
       <c r="Z172" t="n">
-        <v>3.6</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="173">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="Y173" t="inlineStr"/>
       <c r="Z173" t="n">
-        <v>2.75</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="174">
@@ -22143,7 +22143,7 @@
       </c>
       <c r="Y174" t="inlineStr"/>
       <c r="Z174" t="n">
-        <v>3.38</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="175">
@@ -22269,7 +22269,7 @@
       </c>
       <c r="Y175" t="inlineStr"/>
       <c r="Z175" t="n">
-        <v>3.61</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="176">
@@ -22391,7 +22391,7 @@
       </c>
       <c r="Y176" t="inlineStr"/>
       <c r="Z176" t="n">
-        <v>3.5</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="177">
@@ -22513,7 +22513,7 @@
       </c>
       <c r="Y177" t="inlineStr"/>
       <c r="Z177" t="n">
-        <v>2.88</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="178">
@@ -22635,7 +22635,7 @@
       </c>
       <c r="Y178" t="inlineStr"/>
       <c r="Z178" t="n">
-        <v>1.88</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="179">
@@ -22761,7 +22761,7 @@
       </c>
       <c r="Y179" t="inlineStr"/>
       <c r="Z179" t="n">
-        <v>3.18</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="180">
@@ -22887,7 +22887,7 @@
       </c>
       <c r="Y180" t="inlineStr"/>
       <c r="Z180" t="n">
-        <v>1.45</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="181">
@@ -23009,7 +23009,7 @@
       </c>
       <c r="Y181" t="inlineStr"/>
       <c r="Z181" t="n">
-        <v>1.43</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="182">
@@ -23131,7 +23131,7 @@
       </c>
       <c r="Y182" t="inlineStr"/>
       <c r="Z182" t="n">
-        <v>1.41</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="183">
@@ -23257,7 +23257,7 @@
       </c>
       <c r="Y183" t="inlineStr"/>
       <c r="Z183" t="n">
-        <v>1.49</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="184">
@@ -23383,7 +23383,7 @@
       </c>
       <c r="Y184" t="inlineStr"/>
       <c r="Z184" t="n">
-        <v>1.42</v>
+        <v>5.62</v>
       </c>
     </row>
     <row r="185">
@@ -23509,7 +23509,7 @@
       </c>
       <c r="Y185" t="inlineStr"/>
       <c r="Z185" t="n">
-        <v>1.43</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="186">
@@ -23631,7 +23631,7 @@
       </c>
       <c r="Y186" t="inlineStr"/>
       <c r="Z186" t="n">
-        <v>1.46</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="187">
@@ -23757,7 +23757,7 @@
       </c>
       <c r="Y187" t="inlineStr"/>
       <c r="Z187" t="n">
-        <v>1.42</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="188">
@@ -23879,7 +23879,7 @@
       </c>
       <c r="Y188" t="inlineStr"/>
       <c r="Z188" t="n">
-        <v>1.43</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="189">
@@ -24005,7 +24005,7 @@
       </c>
       <c r="Y189" t="inlineStr"/>
       <c r="Z189" t="n">
-        <v>1.47</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="190">
@@ -24127,7 +24127,7 @@
       </c>
       <c r="Y190" t="inlineStr"/>
       <c r="Z190" t="n">
-        <v>1.47</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="191">
@@ -24249,7 +24249,7 @@
       </c>
       <c r="Y191" t="inlineStr"/>
       <c r="Z191" t="n">
-        <v>1.44</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="192">
@@ -24375,7 +24375,7 @@
       </c>
       <c r="Y192" t="inlineStr"/>
       <c r="Z192" t="n">
-        <v>1.45</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="193">
@@ -24497,7 +24497,7 @@
       </c>
       <c r="Y193" t="inlineStr"/>
       <c r="Z193" t="n">
-        <v>1.45</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="194">
@@ -24623,7 +24623,7 @@
       </c>
       <c r="Y194" t="inlineStr"/>
       <c r="Z194" t="n">
-        <v>1.52</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="195">
@@ -24749,7 +24749,7 @@
       </c>
       <c r="Y195" t="inlineStr"/>
       <c r="Z195" t="n">
-        <v>1.43</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="196">
@@ -24871,7 +24871,7 @@
       </c>
       <c r="Y196" t="inlineStr"/>
       <c r="Z196" t="n">
-        <v>1.44</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="197">
@@ -24997,7 +24997,7 @@
       </c>
       <c r="Y197" t="inlineStr"/>
       <c r="Z197" t="n">
-        <v>1.43</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="198">
@@ -25119,7 +25119,7 @@
       </c>
       <c r="Y198" t="inlineStr"/>
       <c r="Z198" t="n">
-        <v>1.44</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="199">
@@ -25241,7 +25241,7 @@
       </c>
       <c r="Y199" t="inlineStr"/>
       <c r="Z199" t="n">
-        <v>1.49</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="200">
@@ -25367,7 +25367,7 @@
       </c>
       <c r="Y200" t="inlineStr"/>
       <c r="Z200" t="n">
-        <v>1.42</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="201">
@@ -25493,7 +25493,7 @@
       </c>
       <c r="Y201" t="inlineStr"/>
       <c r="Z201" t="n">
-        <v>1.45</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="202">
@@ -25619,7 +25619,7 @@
       </c>
       <c r="Y202" t="inlineStr"/>
       <c r="Z202" t="n">
-        <v>1.44</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="203">
@@ -25745,7 +25745,7 @@
       </c>
       <c r="Y203" t="inlineStr"/>
       <c r="Z203" t="n">
-        <v>1.21</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="204">
@@ -25871,7 +25871,7 @@
       </c>
       <c r="Y204" t="inlineStr"/>
       <c r="Z204" t="n">
-        <v>1.81</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="205">
@@ -25993,7 +25993,7 @@
       </c>
       <c r="Y205" t="inlineStr"/>
       <c r="Z205" t="n">
-        <v>1.26</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="206">
@@ -26119,7 +26119,7 @@
       </c>
       <c r="Y206" t="inlineStr"/>
       <c r="Z206" t="n">
-        <v>1.49</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="207">
@@ -26245,7 +26245,7 @@
       </c>
       <c r="Y207" t="inlineStr"/>
       <c r="Z207" t="n">
-        <v>1.23</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="208">
@@ -26371,7 +26371,7 @@
       </c>
       <c r="Y208" t="inlineStr"/>
       <c r="Z208" t="n">
-        <v>1.29</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="209">
@@ -26493,7 +26493,7 @@
       </c>
       <c r="Y209" t="inlineStr"/>
       <c r="Z209" t="n">
-        <v>1.25</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="210">
@@ -26619,7 +26619,7 @@
       </c>
       <c r="Y210" t="inlineStr"/>
       <c r="Z210" t="n">
-        <v>1.42</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="211">
@@ -26745,7 +26745,7 @@
       </c>
       <c r="Y211" t="inlineStr"/>
       <c r="Z211" t="n">
-        <v>1.98</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="212">
@@ -26871,7 +26871,7 @@
       </c>
       <c r="Y212" t="inlineStr"/>
       <c r="Z212" t="n">
-        <v>1.25</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="213">
@@ -26997,7 +26997,7 @@
       </c>
       <c r="Y213" t="inlineStr"/>
       <c r="Z213" t="n">
-        <v>1.24</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="214">
@@ -27123,7 +27123,7 @@
       </c>
       <c r="Y214" t="inlineStr"/>
       <c r="Z214" t="n">
-        <v>1.27</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="215">
@@ -27249,7 +27249,7 @@
       </c>
       <c r="Y215" t="inlineStr"/>
       <c r="Z215" t="n">
-        <v>1.74</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="216">
@@ -27375,7 +27375,7 @@
       </c>
       <c r="Y216" t="inlineStr"/>
       <c r="Z216" t="n">
-        <v>1.26</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="217">
@@ -27501,7 +27501,7 @@
       </c>
       <c r="Y217" t="inlineStr"/>
       <c r="Z217" t="n">
-        <v>1.13</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="218">
@@ -27753,7 +27753,7 @@
       </c>
       <c r="Y219" t="inlineStr"/>
       <c r="Z219" t="n">
-        <v>1.67</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="220">
@@ -27879,7 +27879,7 @@
       </c>
       <c r="Y220" t="inlineStr"/>
       <c r="Z220" t="n">
-        <v>1.16</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="221">
@@ -28001,7 +28001,7 @@
       </c>
       <c r="Y221" t="inlineStr"/>
       <c r="Z221" t="n">
-        <v>1.07</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="222">
@@ -28127,7 +28127,7 @@
       </c>
       <c r="Y222" t="inlineStr"/>
       <c r="Z222" t="n">
-        <v>1.28</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="223">
@@ -28253,7 +28253,7 @@
       </c>
       <c r="Y223" t="inlineStr"/>
       <c r="Z223" t="n">
-        <v>1.8</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="224">
@@ -28379,7 +28379,7 @@
       </c>
       <c r="Y224" t="inlineStr"/>
       <c r="Z224" t="n">
-        <v>1.17</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="225">
@@ -28501,7 +28501,7 @@
       </c>
       <c r="Y225" t="inlineStr"/>
       <c r="Z225" t="n">
-        <v>2.04</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="226">
@@ -28627,7 +28627,7 @@
       </c>
       <c r="Y226" t="inlineStr"/>
       <c r="Z226" t="n">
-        <v>1.19</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="227">
@@ -28753,7 +28753,7 @@
       </c>
       <c r="Y227" t="inlineStr"/>
       <c r="Z227" t="n">
-        <v>1.86</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="228">
@@ -28875,7 +28875,7 @@
       </c>
       <c r="Y228" t="inlineStr"/>
       <c r="Z228" t="n">
-        <v>1.43</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="229">
@@ -29001,7 +29001,7 @@
       </c>
       <c r="Y229" t="inlineStr"/>
       <c r="Z229" t="n">
-        <v>1.46</v>
+        <v>1.28</v>
       </c>
     </row>
     <row r="230">
@@ -29249,7 +29249,7 @@
       </c>
       <c r="Y231" t="inlineStr"/>
       <c r="Z231" t="n">
-        <v>1.02</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="232">
@@ -29371,7 +29371,7 @@
       </c>
       <c r="Y232" t="inlineStr"/>
       <c r="Z232" t="n">
-        <v>1.03</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="233">
@@ -29497,7 +29497,7 @@
       </c>
       <c r="Y233" t="inlineStr"/>
       <c r="Z233" t="n">
-        <v>1.25</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="234">
@@ -29619,7 +29619,7 @@
       </c>
       <c r="Y234" t="inlineStr"/>
       <c r="Z234" t="n">
-        <v>1.79</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="235">
@@ -29745,7 +29745,7 @@
       </c>
       <c r="Y235" t="inlineStr"/>
       <c r="Z235" t="n">
-        <v>1.64</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="236">
@@ -29867,7 +29867,7 @@
       </c>
       <c r="Y236" t="inlineStr"/>
       <c r="Z236" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="237">
@@ -29989,7 +29989,7 @@
       </c>
       <c r="Y237" t="inlineStr"/>
       <c r="Z237" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="238">
@@ -30115,7 +30115,7 @@
       </c>
       <c r="Y238" t="inlineStr"/>
       <c r="Z238" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="239">
@@ -30241,7 +30241,7 @@
       </c>
       <c r="Y239" t="inlineStr"/>
       <c r="Z239" t="n">
-        <v>1.64</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="240">
@@ -30367,7 +30367,7 @@
       </c>
       <c r="Y240" t="inlineStr"/>
       <c r="Z240" t="n">
-        <v>1.22</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="241">
@@ -30493,7 +30493,7 @@
       </c>
       <c r="Y241" t="inlineStr"/>
       <c r="Z241" t="n">
-        <v>2.03</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="242">
@@ -30615,7 +30615,7 @@
       </c>
       <c r="Y242" t="inlineStr"/>
       <c r="Z242" t="n">
-        <v>1.78</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="243">
@@ -30741,7 +30741,7 @@
       </c>
       <c r="Y243" t="inlineStr"/>
       <c r="Z243" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="244">
@@ -30867,7 +30867,7 @@
       </c>
       <c r="Y244" t="inlineStr"/>
       <c r="Z244" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="245">
@@ -30993,7 +30993,7 @@
       </c>
       <c r="Y245" t="inlineStr"/>
       <c r="Z245" t="n">
-        <v>1.2</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="246">
@@ -31115,7 +31115,7 @@
       </c>
       <c r="Y246" t="inlineStr"/>
       <c r="Z246" t="n">
-        <v>1.3</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="247">
@@ -31237,7 +31237,7 @@
       </c>
       <c r="Y247" t="inlineStr"/>
       <c r="Z247" t="n">
-        <v>1.19</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="248">
@@ -31363,7 +31363,7 @@
       </c>
       <c r="Y248" t="inlineStr"/>
       <c r="Z248" t="n">
-        <v>1.12</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="249">
@@ -31489,7 +31489,7 @@
       </c>
       <c r="Y249" t="inlineStr"/>
       <c r="Z249" t="n">
-        <v>1.23</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="250">
@@ -31615,7 +31615,7 @@
       </c>
       <c r="Y250" t="inlineStr"/>
       <c r="Z250" t="n">
-        <v>1.04</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="251">

</xml_diff>